<commit_message>
chore(templates): update BOM Excel template
- Update BomTemplateV3.xlsx binary content

- Align template with current BOM structure
</commit_message>
<xml_diff>
--- a/src/resources/templates/BomTemplateV3.xlsx
+++ b/src/resources/templates/BomTemplateV3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\BomCheck\data\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\BomCheck\src\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F652955D-3843-474D-A1FA-7E47E543F9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D0711F-DFAA-4D93-8299-7280B52E0CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="844" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Sheet1" sheetId="12" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$L$6:$O$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$B$2:$O$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$K$5:$N$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$N$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t xml:space="preserve">Model No: </t>
   </si>
@@ -117,9 +117,6 @@
   </si>
   <si>
     <t>Device Package</t>
-  </si>
-  <si>
-    <t>Build Stage</t>
   </si>
   <si>
     <t>U/P (RMB W/ VAT)</t>
@@ -241,7 +238,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -305,15 +302,18 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -622,248 +622,245 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF954E57-69DF-4516-882C-8CFD4CFAF6E1}">
-  <dimension ref="B2:O10"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3" style="16" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.6640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" style="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.77734375" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" style="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.5546875" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="12.5546875" style="16" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.21875" style="16" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.6640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15" style="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.88671875" style="16" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="27.88671875" style="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="9" style="16"/>
+    <col min="1" max="1" width="4.6640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" style="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.77734375" style="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.5546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.5546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.21875" style="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.6640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" style="16" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.88671875" style="16" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="27.88671875" style="16" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9" style="16"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B2" s="18" t="s">
+    <row r="1" spans="1:14" s="21" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B3" s="20" t="s">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="L2" s="10"/>
+      <c r="M2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N2" s="11">
+        <f>SUM(N3:N4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="18"/>
+      <c r="C3" s="17"/>
       <c r="D3" s="17"/>
       <c r="E3" s="17"/>
       <c r="F3" s="17"/>
       <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="H3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I3" s="17"/>
       <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="M3" s="10"/>
-      <c r="N3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="O3" s="11">
-        <f>SUM(O4:O5)</f>
+      <c r="K3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="L3" s="12"/>
+      <c r="M3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="N3" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="20"/>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="18"/>
+      <c r="C4" s="17"/>
       <c r="D4" s="17"/>
       <c r="E4" s="17"/>
       <c r="F4" s="17"/>
       <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="2" t="s">
-        <v>3</v>
-      </c>
+      <c r="H4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="17"/>
       <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="M4" s="12"/>
-      <c r="N4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="O4" s="11">
+      <c r="K4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="L4" s="10"/>
+      <c r="M4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N4" s="11">
+        <f>SUM(N6:N289)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B5" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="M5" s="10"/>
-      <c r="N5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O5" s="11">
-        <f>SUM(O7:O290)</f>
-        <v>0</v>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>27</v>
-      </c>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="13"/>
       <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
+      <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="15"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="14"/>
       <c r="N7" s="14"/>
-      <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="13"/>
       <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
+      <c r="I8" s="8"/>
       <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="15"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="14"/>
       <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="13"/>
       <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
+      <c r="I9" s="8"/>
       <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="15"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="14"/>
       <c r="N9" s="14"/>
-      <c r="O9" s="14"/>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="15"/>
-      <c r="N10" s="14"/>
-      <c r="O10" s="14"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="11">
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="C4:G4"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.118055555555556" right="0.196527777777778" top="0.196527777777778" bottom="0.118055555555556" header="0.15625" footer="0.118055555555556"/>

</xml_diff>